<commit_message>
Add invariance guardrails and unify the suite
</commit_message>
<xml_diff>
--- a/examples/measuresignal-starter-template.xlsx
+++ b/examples/measuresignal-starter-template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Response data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response data'!$A$1:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response data'!$A$1:$J$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,11 +427,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -439,6 +439,7 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,40 +450,45 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>collection_wave</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>item_1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>item_2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>item_3</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>item_4</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>item_5</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>item_6</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>item_7</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>item_8</t>
         </is>
@@ -494,7 +500,11 @@
           <t>R001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
@@ -502,6 +512,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -509,7 +520,11 @@
           <t>R002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
@@ -517,6 +532,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -524,7 +540,11 @@
           <t>R003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
@@ -532,6 +552,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -539,7 +560,11 @@
           <t>R004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
@@ -547,6 +572,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -554,7 +580,11 @@
           <t>R005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
@@ -562,6 +592,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -569,7 +600,11 @@
           <t>R006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
@@ -577,6 +612,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -584,7 +620,11 @@
           <t>R007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
@@ -592,6 +632,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -599,7 +640,11 @@
           <t>R008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
@@ -607,6 +652,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -614,7 +660,11 @@
           <t>R009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
@@ -622,6 +672,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -629,7 +680,11 @@
           <t>R010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
@@ -637,6 +692,7 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -644,7 +700,11 @@
           <t>R011</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
@@ -652,6 +712,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -659,7 +720,11 @@
           <t>R012</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
@@ -667,9 +732,10 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I13"/>
+  <autoFilter ref="A1:J13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>